<commit_message>
Support sample-sheet barcode matching and compressed workflow exports
</commit_message>
<xml_diff>
--- a/example/reference_results/1_data_integrity_and_sample_mapping/data_integrity_and_sample_mapping.xlsx
+++ b/example/reference_results/1_data_integrity_and_sample_mapping/data_integrity_and_sample_mapping.xlsx
@@ -8,7 +8,7 @@
   <sheets>
     <sheet name="Run_Summary" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="Sample_Manifest" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Archive_Inventory" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="FASTQ_Inventory" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="Column_Dictionary" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
 </workbook>
@@ -52,7 +52,7 @@
             <color rgb="FF000000"/>
             <name val="Tahoma"/>
           </rPr>
-          <t xml:space="preserve">Number of FASTQ ZIP archives discovered for the pool.</t>
+          <t xml:space="preserve">Number of compressed FASTQ files discovered in the pool.</t>
         </r>
       </text>
     </comment>
@@ -64,7 +64,7 @@
             <color rgb="FF000000"/>
             <name val="Tahoma"/>
           </rPr>
-          <t xml:space="preserve">Filename of the validated FASTQ ZIP archive for the pool.</t>
+          <t xml:space="preserve">Number of sample-sheet rows belonging to supplied pools; stored as a numeric Excel value.</t>
         </r>
       </text>
     </comment>
@@ -76,7 +76,7 @@
             <color rgb="FF000000"/>
             <name val="Tahoma"/>
           </rPr>
-          <t xml:space="preserve">Number of recognized FASTQ members delivered in the pool archive.</t>
+          <t xml:space="preserve">Number of active samples matched to exactly one supplied file; stored as a numeric Excel value.</t>
         </r>
       </text>
     </comment>
@@ -88,7 +88,7 @@
             <color rgb="FF000000"/>
             <name val="Tahoma"/>
           </rPr>
-          <t xml:space="preserve">Number of sample-sheet rows belonging to supplied pools; stored as a numeric Excel value.</t>
+          <t xml:space="preserve">Number of copied FASTQ files that parsed completely; stored as a numeric Excel value.</t>
         </r>
       </text>
     </comment>
@@ -100,7 +100,7 @@
             <color rgb="FF000000"/>
             <name val="Tahoma"/>
           </rPr>
-          <t xml:space="preserve">Number of active samples matched to exactly one archive member; stored as a numeric Excel value.</t>
+          <t xml:space="preserve">Total FASTQ records across all mapped samples; stored as a numeric Excel value.</t>
         </r>
       </text>
     </comment>
@@ -112,7 +112,7 @@
             <color rgb="FF000000"/>
             <name val="Tahoma"/>
           </rPr>
-          <t xml:space="preserve">Number of extracted FASTQ files that parsed completely; stored as a numeric Excel value.</t>
+          <t xml:space="preserve">Pool-level PASS only when every active sample maps and every mapped FASTQ validates.</t>
         </r>
       </text>
     </comment>
@@ -124,31 +124,7 @@
             <color rgb="FF000000"/>
             <name val="Tahoma"/>
           </rPr>
-          <t xml:space="preserve">Total FASTQ records across all mapped samples; stored as a numeric Excel value.</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="J1" authorId="0" shapeId="0">
-      <text>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <color rgb="FF000000"/>
-            <name val="Tahoma"/>
-          </rPr>
-          <t xml:space="preserve">Archive members not listed in the active sample sheet; stored as a numeric Excel value.</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="K1" authorId="0" shapeId="0">
-      <text>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <color rgb="FF000000"/>
-            <name val="Tahoma"/>
-          </rPr>
-          <t xml:space="preserve">Pool-level PASS only when every active sample maps and every mapped FASTQ validates.</t>
+          <t xml:space="preserve">Delivered FASTQ files not requested by the active sample sheet.</t>
         </r>
       </text>
     </comment>
@@ -206,7 +182,7 @@
             <color rgb="FF000000"/>
             <name val="Tahoma"/>
           </rPr>
-          <t xml:space="preserve">Forward Lima barcode identifier used in the pool-specific mapping key.</t>
+          <t xml:space="preserve">Forward barcode identifier supplied in the sample sheet used in the pool-specific mapping key.</t>
         </r>
       </text>
     </comment>
@@ -218,7 +194,7 @@
             <color rgb="FF000000"/>
             <name val="Tahoma"/>
           </rPr>
-          <t xml:space="preserve">Reverse Lima barcode identifier used in the pool-specific mapping key.</t>
+          <t xml:space="preserve">Reverse barcode identifier supplied in the sample sheet used in the pool-specific mapping key.</t>
         </r>
       </text>
     </comment>
@@ -230,7 +206,7 @@
             <color rgb="FF000000"/>
             <name val="Tahoma"/>
           </rPr>
-          <t xml:space="preserve">Quality label embedded in the delivered Lima filename, such as Q20; this is not recalculated here.</t>
+          <t xml:space="preserve">Original compressed FASTQ filename within the pool directory.</t>
         </r>
       </text>
     </comment>
@@ -242,7 +218,7 @@
             <color rgb="FF000000"/>
             <name val="Tahoma"/>
           </rPr>
-          <t xml:space="preserve">Filename of the immutable raw PacBio FASTQ ZIP archive.</t>
+          <t xml:space="preserve">Workflow-ready sample FASTQ path created by this notebook under mapped_fastq/.</t>
         </r>
       </text>
     </comment>
@@ -254,7 +230,7 @@
             <color rgb="FF000000"/>
             <name val="Tahoma"/>
           </rPr>
-          <t xml:space="preserve">Original pool-demultiplexed FASTQ member path inside the ZIP archive.</t>
+          <t xml:space="preserve">Number of completely parsed FASTQ records in the copied sample file.</t>
         </r>
       </text>
     </comment>
@@ -266,7 +242,7 @@
             <color rgb="FF000000"/>
             <name val="Tahoma"/>
           </rPr>
-          <t xml:space="preserve">Workflow-ready sample FASTQ path created by this notebook under mapped_fastq/.</t>
+          <t xml:space="preserve">Copied FASTQ file size in mebibytes, rounded to three decimal places.</t>
         </r>
       </text>
     </comment>
@@ -278,31 +254,7 @@
             <color rgb="FF000000"/>
             <name val="Tahoma"/>
           </rPr>
-          <t xml:space="preserve">Number of completely parsed FASTQ records in the extracted sample file.</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="K1" authorId="0" shapeId="0">
-      <text>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <color rgb="FF000000"/>
-            <name val="Tahoma"/>
-          </rPr>
-          <t xml:space="preserve">Extracted FASTQ file size in mebibytes, rounded to three decimal places.</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="L1" authorId="0" shapeId="0">
-      <text>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <color rgb="FF000000"/>
-            <name val="Tahoma"/>
-          </rPr>
-          <t xml:space="preserve">PASS when sample mapping succeeded and the complete extracted FASTQ parsed without error.</t>
+          <t xml:space="preserve">PASS when sample mapping succeeded and the complete copied FASTQ parsed without error.</t>
         </r>
       </text>
     </comment>
@@ -336,7 +288,7 @@
             <color rgb="FF000000"/>
             <name val="Tahoma"/>
           </rPr>
-          <t xml:space="preserve">Filename of the immutable raw PacBio FASTQ ZIP archive.</t>
+          <t xml:space="preserve">Original compressed FASTQ filename within the pool directory.</t>
         </r>
       </text>
     </comment>
@@ -348,59 +300,11 @@
             <color rgb="FF000000"/>
             <name val="Tahoma"/>
           </rPr>
-          <t xml:space="preserve">Original pool-demultiplexed FASTQ member path inside the ZIP archive.</t>
+          <t xml:space="preserve">Delivered gzip FASTQ size in bytes.</t>
         </r>
       </text>
     </comment>
     <comment ref="D1" authorId="0" shapeId="0">
-      <text>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <color rgb="FF000000"/>
-            <name val="Tahoma"/>
-          </rPr>
-          <t xml:space="preserve">Forward Lima barcode identifier used in the pool-specific mapping key.</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="E1" authorId="0" shapeId="0">
-      <text>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <color rgb="FF000000"/>
-            <name val="Tahoma"/>
-          </rPr>
-          <t xml:space="preserve">Reverse Lima barcode identifier used in the pool-specific mapping key.</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="F1" authorId="0" shapeId="0">
-      <text>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <color rgb="FF000000"/>
-            <name val="Tahoma"/>
-          </rPr>
-          <t xml:space="preserve">Quality label embedded in the delivered Lima filename, such as Q20; this is not recalculated here.</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="G1" authorId="0" shapeId="0">
-      <text>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <color rgb="FF000000"/>
-            <name val="Tahoma"/>
-          </rPr>
-          <t xml:space="preserve">Uncompressed member size reported by the ZIP directory.</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="H1" authorId="0" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -463,7 +367,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="75" uniqueCount="75">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="64" uniqueCount="64">
   <si>
     <t xml:space="preserve">PoolNumber</t>
   </si>
@@ -471,13 +375,7 @@
     <t xml:space="preserve">PoolDirectory</t>
   </si>
   <si>
-    <t xml:space="preserve">ArchiveCount</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ArchiveFile</t>
-  </si>
-  <si>
-    <t xml:space="preserve">FASTQMemberCount</t>
+    <t xml:space="preserve">FASTQFileCount</t>
   </si>
   <si>
     <t xml:space="preserve">ActiveSampleCount</t>
@@ -492,18 +390,15 @@
     <t xml:space="preserve">TotalInputReads</t>
   </si>
   <si>
-    <t xml:space="preserve">UnlistedArchiveMemberCount</t>
-  </si>
-  <si>
     <t xml:space="preserve">OverallStatus</t>
   </si>
   <si>
+    <t xml:space="preserve">UnlistedFASTQCount</t>
+  </si>
+  <si>
     <t xml:space="preserve">pool1</t>
   </si>
   <si>
-    <t xml:space="preserve">Callahan-Fecal-HiFi-Example.fastq.zip</t>
-  </si>
-  <si>
     <t xml:space="preserve">PASS</t>
   </si>
   <si>
@@ -519,13 +414,7 @@
     <t xml:space="preserve">ReverseBarcodeID</t>
   </si>
   <si>
-    <t xml:space="preserve">LimaQualityLabel</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SourceArchive</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ArchiveMember</t>
+    <t xml:space="preserve">SourceFASTQ</t>
   </si>
   <si>
     <t xml:space="preserve">MappedFASTQ</t>
@@ -546,13 +435,10 @@
     <t xml:space="preserve">bc1004</t>
   </si>
   <si>
-    <t xml:space="preserve">Q20</t>
-  </si>
-  <si>
-    <t xml:space="preserve">lima.bc1004--bc1004.Q20.fastq</t>
-  </si>
-  <si>
-    <t xml:space="preserve">/Users/amro/Documents/workflows/DADA2_16S_PacBio_HiFi_Workflow/example/run_results/1_data_integrity_and_sample_mapping/mapped_fastq/Subject-R11-Timepoint-1.fastq</t>
+    <t xml:space="preserve">lima.bc1004--bc1004.Q20.fastq.gz</t>
+  </si>
+  <si>
+    <t xml:space="preserve">/Users/amro/Documents/workflows/DADA2_16S_PacBio_HiFi_Workflow/example/run_results/1_data_integrity_and_sample_mapping/mapped_fastq/Subject-R11-Timepoint-1.fastq.gz</t>
   </si>
   <si>
     <t xml:space="preserve">Subject-R3-Timepoint-1</t>
@@ -561,10 +447,10 @@
     <t xml:space="preserve">bc1001</t>
   </si>
   <si>
-    <t xml:space="preserve">lima.bc1001--bc1001.Q20.fastq</t>
-  </si>
-  <si>
-    <t xml:space="preserve">/Users/amro/Documents/workflows/DADA2_16S_PacBio_HiFi_Workflow/example/run_results/1_data_integrity_and_sample_mapping/mapped_fastq/Subject-R3-Timepoint-1.fastq</t>
+    <t xml:space="preserve">lima.bc1001--bc1001.Q20.fastq.gz</t>
+  </si>
+  <si>
+    <t xml:space="preserve">/Users/amro/Documents/workflows/DADA2_16S_PacBio_HiFi_Workflow/example/run_results/1_data_integrity_and_sample_mapping/mapped_fastq/Subject-R3-Timepoint-1.fastq.gz</t>
   </si>
   <si>
     <t xml:space="preserve">Subject-R3-Timepoint-2</t>
@@ -573,10 +459,10 @@
     <t xml:space="preserve">bc1002</t>
   </si>
   <si>
-    <t xml:space="preserve">lima.bc1002--bc1002.Q20.fastq</t>
-  </si>
-  <si>
-    <t xml:space="preserve">/Users/amro/Documents/workflows/DADA2_16S_PacBio_HiFi_Workflow/example/run_results/1_data_integrity_and_sample_mapping/mapped_fastq/Subject-R3-Timepoint-2.fastq</t>
+    <t xml:space="preserve">lima.bc1002--bc1002.Q20.fastq.gz</t>
+  </si>
+  <si>
+    <t xml:space="preserve">/Users/amro/Documents/workflows/DADA2_16S_PacBio_HiFi_Workflow/example/run_results/1_data_integrity_and_sample_mapping/mapped_fastq/Subject-R3-Timepoint-2.fastq.gz</t>
   </si>
   <si>
     <t xml:space="preserve">Subject-R3-Timepoint-3</t>
@@ -585,16 +471,13 @@
     <t xml:space="preserve">bc1003</t>
   </si>
   <si>
-    <t xml:space="preserve">lima.bc1003--bc1003.Q20.fastq</t>
-  </si>
-  <si>
-    <t xml:space="preserve">/Users/amro/Documents/workflows/DADA2_16S_PacBio_HiFi_Workflow/example/run_results/1_data_integrity_and_sample_mapping/mapped_fastq/Subject-R3-Timepoint-3.fastq</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Archive</t>
-  </si>
-  <si>
-    <t xml:space="preserve">UncompressedSizeBytes</t>
+    <t xml:space="preserve">lima.bc1003--bc1003.Q20.fastq.gz</t>
+  </si>
+  <si>
+    <t xml:space="preserve">/Users/amro/Documents/workflows/DADA2_16S_PacBio_HiFi_Workflow/example/run_results/1_data_integrity_and_sample_mapping/mapped_fastq/Subject-R3-Timepoint-3.fastq.gz</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CompressedSizeBytes</t>
   </si>
   <si>
     <t xml:space="preserve">ListedInSampleSheet</t>
@@ -618,33 +501,27 @@
     <t xml:space="preserve">Pool directory name discovered under data/fastq/.</t>
   </si>
   <si>
-    <t xml:space="preserve">Number of FASTQ ZIP archives discovered for the pool.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Filename of the validated FASTQ ZIP archive for the pool.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Number of recognized FASTQ members delivered in the pool archive.</t>
+    <t xml:space="preserve">Number of compressed FASTQ files discovered in the pool.</t>
   </si>
   <si>
     <t xml:space="preserve">Number of sample-sheet rows belonging to supplied pools; stored as a numeric Excel value.</t>
   </si>
   <si>
-    <t xml:space="preserve">Number of active samples matched to exactly one archive member; stored as a numeric Excel value.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Number of extracted FASTQ files that parsed completely; stored as a numeric Excel value.</t>
+    <t xml:space="preserve">Number of active samples matched to exactly one supplied file; stored as a numeric Excel value.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Number of copied FASTQ files that parsed completely; stored as a numeric Excel value.</t>
   </si>
   <si>
     <t xml:space="preserve">Total FASTQ records across all mapped samples; stored as a numeric Excel value.</t>
   </si>
   <si>
-    <t xml:space="preserve">Archive members not listed in the active sample sheet; stored as a numeric Excel value.</t>
-  </si>
-  <si>
     <t xml:space="preserve">Pool-level PASS only when every active sample maps and every mapped FASTQ validates.</t>
   </si>
   <si>
+    <t xml:space="preserve">Delivered FASTQ files not requested by the active sample sheet.</t>
+  </si>
+  <si>
     <t xml:space="preserve">Sample_Manifest</t>
   </si>
   <si>
@@ -654,37 +531,31 @@
     <t xml:space="preserve">Biological sample identifier exactly as recorded in data/sample_sheet.xlsx before filename-safe sanitization.</t>
   </si>
   <si>
-    <t xml:space="preserve">Forward Lima barcode identifier used in the pool-specific mapping key.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Reverse Lima barcode identifier used in the pool-specific mapping key.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Quality label embedded in the delivered Lima filename, such as Q20; this is not recalculated here.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Filename of the immutable raw PacBio FASTQ ZIP archive.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Original pool-demultiplexed FASTQ member path inside the ZIP archive.</t>
+    <t xml:space="preserve">Forward barcode identifier supplied in the sample sheet used in the pool-specific mapping key.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Reverse barcode identifier supplied in the sample sheet used in the pool-specific mapping key.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Original compressed FASTQ filename within the pool directory.</t>
   </si>
   <si>
     <t xml:space="preserve">Workflow-ready sample FASTQ path created by this notebook under mapped_fastq/.</t>
   </si>
   <si>
-    <t xml:space="preserve">Number of completely parsed FASTQ records in the extracted sample file.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Extracted FASTQ file size in mebibytes, rounded to three decimal places.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">PASS when sample mapping succeeded and the complete extracted FASTQ parsed without error.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Archive_Inventory</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Uncompressed member size reported by the ZIP directory.</t>
+    <t xml:space="preserve">Number of completely parsed FASTQ records in the copied sample file.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Copied FASTQ file size in mebibytes, rounded to three decimal places.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PASS when sample mapping succeeded and the complete copied FASTQ parsed without error.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">FASTQ_Inventory</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Delivered gzip FASTQ size in bytes.</t>
   </si>
   <si>
     <t xml:space="preserve">Whether the pool/barcode pair appears in a sample-sheet row for a supplied pool.</t>
@@ -744,66 +615,58 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="Table3" displayName="Table3" ref="A1:K2" totalsRowCount="0" totalsRowShown="0">
-  <autoFilter ref="A1:K2"/>
-  <tableColumns count="11">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="Table3" displayName="Table3" ref="A1:I2" totalsRowCount="0" totalsRowShown="0">
+  <autoFilter ref="A1:I2"/>
+  <tableColumns count="9">
     <tableColumn id="1" name="PoolNumber"/>
     <tableColumn id="2" name="PoolDirectory"/>
-    <tableColumn id="3" name="ArchiveCount"/>
-    <tableColumn id="4" name="ArchiveFile"/>
-    <tableColumn id="5" name="FASTQMemberCount"/>
-    <tableColumn id="6" name="ActiveSampleCount"/>
-    <tableColumn id="7" name="MatchedSampleCount"/>
-    <tableColumn id="8" name="ValidFASTQCount"/>
-    <tableColumn id="9" name="TotalInputReads"/>
-    <tableColumn id="10" name="UnlistedArchiveMemberCount"/>
-    <tableColumn id="11" name="OverallStatus"/>
+    <tableColumn id="3" name="FASTQFileCount"/>
+    <tableColumn id="4" name="ActiveSampleCount"/>
+    <tableColumn id="5" name="MatchedSampleCount"/>
+    <tableColumn id="6" name="ValidFASTQCount"/>
+    <tableColumn id="7" name="TotalInputReads"/>
+    <tableColumn id="8" name="OverallStatus"/>
+    <tableColumn id="9" name="UnlistedFASTQCount"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight9" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="Table4" displayName="Table4" ref="A1:L5" totalsRowCount="0" totalsRowShown="0">
-  <autoFilter ref="A1:L5"/>
-  <tableColumns count="12">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="Table4" displayName="Table4" ref="A1:J5" totalsRowCount="0" totalsRowShown="0">
+  <autoFilter ref="A1:J5"/>
+  <tableColumns count="10">
     <tableColumn id="1" name="PoolNumber"/>
     <tableColumn id="2" name="SampleID"/>
     <tableColumn id="3" name="SourceSampleID"/>
     <tableColumn id="4" name="ForwardBarcodeID"/>
     <tableColumn id="5" name="ReverseBarcodeID"/>
-    <tableColumn id="6" name="LimaQualityLabel"/>
-    <tableColumn id="7" name="SourceArchive"/>
-    <tableColumn id="8" name="ArchiveMember"/>
-    <tableColumn id="9" name="MappedFASTQ"/>
-    <tableColumn id="10" name="InputReads"/>
-    <tableColumn id="11" name="OutputSizeMB"/>
-    <tableColumn id="12" name="IntegrityStatus"/>
+    <tableColumn id="6" name="SourceFASTQ"/>
+    <tableColumn id="7" name="MappedFASTQ"/>
+    <tableColumn id="8" name="InputReads"/>
+    <tableColumn id="9" name="OutputSizeMB"/>
+    <tableColumn id="10" name="IntegrityStatus"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight9" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="Table5" displayName="Table5" ref="A1:H5" totalsRowCount="0" totalsRowShown="0">
-  <autoFilter ref="A1:H5"/>
-  <tableColumns count="8">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="Table5" displayName="Table5" ref="A1:D5" totalsRowCount="0" totalsRowShown="0">
+  <autoFilter ref="A1:D5"/>
+  <tableColumns count="4">
     <tableColumn id="1" name="PoolNumber"/>
-    <tableColumn id="2" name="Archive"/>
-    <tableColumn id="3" name="ArchiveMember"/>
-    <tableColumn id="4" name="ForwardBarcodeID"/>
-    <tableColumn id="5" name="ReverseBarcodeID"/>
-    <tableColumn id="6" name="LimaQualityLabel"/>
-    <tableColumn id="7" name="UncompressedSizeBytes"/>
-    <tableColumn id="8" name="ListedInSampleSheet"/>
+    <tableColumn id="2" name="SourceFASTQ"/>
+    <tableColumn id="3" name="CompressedSizeBytes"/>
+    <tableColumn id="4" name="ListedInSampleSheet"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight9" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="6" name="Table6" displayName="Table6" ref="A1:C32" totalsRowCount="0" totalsRowShown="0">
-  <autoFilter ref="A1:C32"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="6" name="Table6" displayName="Table6" ref="A1:C24" totalsRowCount="0" totalsRowShown="0">
+  <autoFilter ref="A1:C24"/>
   <tableColumns count="3">
     <tableColumn id="1" name="Sheet"/>
     <tableColumn id="2" name="Column"/>
@@ -1100,15 +963,13 @@
   <cols>
     <col min="1" max="1" width="10.71" hidden="0" customWidth="1"/>
     <col min="2" max="2" width="13.71" hidden="0" customWidth="1"/>
-    <col min="3" max="3" width="12.71" hidden="0" customWidth="1"/>
-    <col min="4" max="4" width="37.71" hidden="0" customWidth="1"/>
-    <col min="5" max="5" width="16.71" hidden="0" customWidth="1"/>
-    <col min="6" max="6" width="17.71" hidden="0" customWidth="1"/>
-    <col min="7" max="7" width="18.71" hidden="0" customWidth="1"/>
-    <col min="8" max="8" width="15.71" hidden="0" customWidth="1"/>
-    <col min="9" max="9" width="15.71" hidden="0" customWidth="1"/>
-    <col min="10" max="10" width="26.71" hidden="0" customWidth="1"/>
-    <col min="11" max="11" width="13.71" hidden="0" customWidth="1"/>
+    <col min="3" max="3" width="14.71" hidden="0" customWidth="1"/>
+    <col min="4" max="4" width="17.71" hidden="0" customWidth="1"/>
+    <col min="5" max="5" width="18.71" hidden="0" customWidth="1"/>
+    <col min="6" max="6" width="15.71" hidden="0" customWidth="1"/>
+    <col min="7" max="7" width="15.71" hidden="0" customWidth="1"/>
+    <col min="8" max="8" width="13.71" hidden="0" customWidth="1"/>
+    <col min="9" max="9" width="18.71" hidden="0" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1139,25 +1000,19 @@
       <c r="I1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="K1" s="1" t="s">
-        <v>10</v>
-      </c>
     </row>
     <row r="2">
       <c r="A2" t="n">
         <v>1</v>
       </c>
       <c r="B2" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="C2" t="n">
-        <v>1</v>
-      </c>
-      <c r="D2" t="s">
-        <v>12</v>
+        <v>4</v>
+      </c>
+      <c r="D2" t="n">
+        <v>4</v>
       </c>
       <c r="E2" t="n">
         <v>4</v>
@@ -1166,19 +1021,13 @@
         <v>4</v>
       </c>
       <c r="G2" t="n">
-        <v>4</v>
-      </c>
-      <c r="H2" t="n">
-        <v>4</v>
+        <v>20000</v>
+      </c>
+      <c r="H2" t="s">
+        <v>10</v>
       </c>
       <c r="I2" t="n">
-        <v>20000</v>
-      </c>
-      <c r="J2" t="n">
         <v>0</v>
-      </c>
-      <c r="K2" t="s">
-        <v>13</v>
       </c>
     </row>
   </sheetData>
@@ -1204,13 +1053,11 @@
     <col min="3" max="3" width="23.71" hidden="0" customWidth="1"/>
     <col min="4" max="4" width="16.71" hidden="0" customWidth="1"/>
     <col min="5" max="5" width="16.71" hidden="0" customWidth="1"/>
-    <col min="6" max="6" width="16.71" hidden="0" customWidth="1"/>
-    <col min="7" max="7" width="37.71" hidden="0" customWidth="1"/>
-    <col min="8" max="8" width="29.71" hidden="0" customWidth="1"/>
-    <col min="9" max="9" width="161.71" hidden="0" customWidth="1"/>
-    <col min="10" max="10" width="10.71" hidden="0" customWidth="1"/>
-    <col min="11" max="11" width="12.71" hidden="0" customWidth="1"/>
-    <col min="12" max="12" width="15.71" hidden="0" customWidth="1"/>
+    <col min="6" max="6" width="32.71" hidden="0" customWidth="1"/>
+    <col min="7" max="7" width="164.71" hidden="0" customWidth="1"/>
+    <col min="8" max="8" width="10.71" hidden="0" customWidth="1"/>
+    <col min="9" max="9" width="12.71" hidden="0" customWidth="1"/>
+    <col min="10" max="10" width="15.71" hidden="0" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1218,37 +1065,31 @@
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="E1" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="F1" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="G1" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="H1" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="I1" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="J1" s="1" t="s">
         <v>19</v>
-      </c>
-      <c r="H1" s="1" t="s">
-        <v>20</v>
-      </c>
-      <c r="I1" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="J1" s="1" t="s">
-        <v>22</v>
-      </c>
-      <c r="K1" s="1" t="s">
-        <v>23</v>
-      </c>
-      <c r="L1" s="1" t="s">
-        <v>24</v>
       </c>
     </row>
     <row r="2">
@@ -1256,37 +1097,31 @@
         <v>1</v>
       </c>
       <c r="B2" t="s">
-        <v>25</v>
+        <v>20</v>
       </c>
       <c r="C2" t="s">
-        <v>25</v>
+        <v>20</v>
       </c>
       <c r="D2" t="s">
-        <v>26</v>
+        <v>21</v>
       </c>
       <c r="E2" t="s">
-        <v>26</v>
+        <v>21</v>
       </c>
       <c r="F2" t="s">
-        <v>27</v>
+        <v>22</v>
       </c>
       <c r="G2" t="s">
-        <v>12</v>
-      </c>
-      <c r="H2" t="s">
-        <v>28</v>
-      </c>
-      <c r="I2" t="s">
-        <v>29</v>
-      </c>
-      <c r="J2" t="n">
+        <v>23</v>
+      </c>
+      <c r="H2" t="n">
         <v>5000</v>
       </c>
-      <c r="K2" t="n">
-        <v>14.431</v>
-      </c>
-      <c r="L2" t="s">
-        <v>13</v>
+      <c r="I2" t="n">
+        <v>1.316</v>
+      </c>
+      <c r="J2" t="s">
+        <v>10</v>
       </c>
     </row>
     <row r="3">
@@ -1294,37 +1129,31 @@
         <v>1</v>
       </c>
       <c r="B3" t="s">
-        <v>30</v>
+        <v>24</v>
       </c>
       <c r="C3" t="s">
-        <v>30</v>
+        <v>24</v>
       </c>
       <c r="D3" t="s">
-        <v>31</v>
+        <v>25</v>
       </c>
       <c r="E3" t="s">
-        <v>31</v>
+        <v>25</v>
       </c>
       <c r="F3" t="s">
+        <v>26</v>
+      </c>
+      <c r="G3" t="s">
         <v>27</v>
       </c>
-      <c r="G3" t="s">
-        <v>12</v>
-      </c>
-      <c r="H3" t="s">
-        <v>32</v>
-      </c>
-      <c r="I3" t="s">
-        <v>33</v>
-      </c>
-      <c r="J3" t="n">
+      <c r="H3" t="n">
         <v>5000</v>
       </c>
-      <c r="K3" t="n">
-        <v>14.38</v>
-      </c>
-      <c r="L3" t="s">
-        <v>13</v>
+      <c r="I3" t="n">
+        <v>1.25</v>
+      </c>
+      <c r="J3" t="s">
+        <v>10</v>
       </c>
     </row>
     <row r="4">
@@ -1332,37 +1161,31 @@
         <v>1</v>
       </c>
       <c r="B4" t="s">
-        <v>34</v>
+        <v>28</v>
       </c>
       <c r="C4" t="s">
-        <v>34</v>
+        <v>28</v>
       </c>
       <c r="D4" t="s">
-        <v>35</v>
+        <v>29</v>
       </c>
       <c r="E4" t="s">
-        <v>35</v>
+        <v>29</v>
       </c>
       <c r="F4" t="s">
-        <v>27</v>
+        <v>30</v>
       </c>
       <c r="G4" t="s">
-        <v>12</v>
-      </c>
-      <c r="H4" t="s">
-        <v>36</v>
-      </c>
-      <c r="I4" t="s">
-        <v>37</v>
-      </c>
-      <c r="J4" t="n">
+        <v>31</v>
+      </c>
+      <c r="H4" t="n">
         <v>5000</v>
       </c>
-      <c r="K4" t="n">
-        <v>14.565</v>
-      </c>
-      <c r="L4" t="s">
-        <v>13</v>
+      <c r="I4" t="n">
+        <v>1.43</v>
+      </c>
+      <c r="J4" t="s">
+        <v>10</v>
       </c>
     </row>
     <row r="5">
@@ -1370,37 +1193,31 @@
         <v>1</v>
       </c>
       <c r="B5" t="s">
-        <v>38</v>
+        <v>32</v>
       </c>
       <c r="C5" t="s">
-        <v>38</v>
+        <v>32</v>
       </c>
       <c r="D5" t="s">
-        <v>39</v>
+        <v>33</v>
       </c>
       <c r="E5" t="s">
-        <v>39</v>
+        <v>33</v>
       </c>
       <c r="F5" t="s">
-        <v>27</v>
+        <v>34</v>
       </c>
       <c r="G5" t="s">
-        <v>12</v>
-      </c>
-      <c r="H5" t="s">
-        <v>40</v>
-      </c>
-      <c r="I5" t="s">
-        <v>41</v>
-      </c>
-      <c r="J5" t="n">
+        <v>35</v>
+      </c>
+      <c r="H5" t="n">
         <v>5000</v>
       </c>
-      <c r="K5" t="n">
-        <v>14.518</v>
-      </c>
-      <c r="L5" t="s">
-        <v>13</v>
+      <c r="I5" t="n">
+        <v>1.32</v>
+      </c>
+      <c r="J5" t="s">
+        <v>10</v>
       </c>
     </row>
   </sheetData>
@@ -1422,13 +1239,9 @@
   <sheetFormatPr defaultRowHeight="15.0" baseColWidth="10"/>
   <cols>
     <col min="1" max="1" width="10.71" hidden="0" customWidth="1"/>
-    <col min="2" max="2" width="37.71" hidden="0" customWidth="1"/>
-    <col min="3" max="3" width="29.71" hidden="0" customWidth="1"/>
-    <col min="4" max="4" width="16.71" hidden="0" customWidth="1"/>
-    <col min="5" max="5" width="16.71" hidden="0" customWidth="1"/>
-    <col min="6" max="6" width="16.71" hidden="0" customWidth="1"/>
-    <col min="7" max="7" width="21.71" hidden="0" customWidth="1"/>
-    <col min="8" max="8" width="19.71" hidden="0" customWidth="1"/>
+    <col min="2" max="2" width="32.71" hidden="0" customWidth="1"/>
+    <col min="3" max="3" width="19.71" hidden="0" customWidth="1"/>
+    <col min="4" max="4" width="19.71" hidden="0" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1436,25 +1249,13 @@
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>42</v>
+        <v>15</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>20</v>
+        <v>36</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>16</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="F1" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="G1" s="1" t="s">
-        <v>43</v>
-      </c>
-      <c r="H1" s="1" t="s">
-        <v>44</v>
+        <v>37</v>
       </c>
     </row>
     <row r="2">
@@ -1462,24 +1263,12 @@
         <v>1</v>
       </c>
       <c r="B2" t="s">
-        <v>12</v>
-      </c>
-      <c r="C2" t="s">
-        <v>32</v>
-      </c>
-      <c r="D2" t="s">
-        <v>31</v>
-      </c>
-      <c r="E2" t="s">
-        <v>31</v>
-      </c>
-      <c r="F2" t="s">
-        <v>27</v>
-      </c>
-      <c r="G2" t="n">
-        <v>15078512</v>
-      </c>
-      <c r="H2" t="b">
+        <v>26</v>
+      </c>
+      <c r="C2" t="n">
+        <v>1310346</v>
+      </c>
+      <c r="D2" t="b">
         <v>1</v>
       </c>
     </row>
@@ -1488,24 +1277,12 @@
         <v>1</v>
       </c>
       <c r="B3" t="s">
-        <v>12</v>
-      </c>
-      <c r="C3" t="s">
-        <v>36</v>
-      </c>
-      <c r="D3" t="s">
-        <v>35</v>
-      </c>
-      <c r="E3" t="s">
-        <v>35</v>
-      </c>
-      <c r="F3" t="s">
-        <v>27</v>
-      </c>
-      <c r="G3" t="n">
-        <v>15272274</v>
-      </c>
-      <c r="H3" t="b">
+        <v>30</v>
+      </c>
+      <c r="C3" t="n">
+        <v>1499078</v>
+      </c>
+      <c r="D3" t="b">
         <v>1</v>
       </c>
     </row>
@@ -1514,24 +1291,12 @@
         <v>1</v>
       </c>
       <c r="B4" t="s">
-        <v>12</v>
-      </c>
-      <c r="C4" t="s">
-        <v>40</v>
-      </c>
-      <c r="D4" t="s">
-        <v>39</v>
-      </c>
-      <c r="E4" t="s">
-        <v>39</v>
-      </c>
-      <c r="F4" t="s">
-        <v>27</v>
-      </c>
-      <c r="G4" t="n">
-        <v>15222900</v>
-      </c>
-      <c r="H4" t="b">
+        <v>34</v>
+      </c>
+      <c r="C4" t="n">
+        <v>1383840</v>
+      </c>
+      <c r="D4" t="b">
         <v>1</v>
       </c>
     </row>
@@ -1540,24 +1305,12 @@
         <v>1</v>
       </c>
       <c r="B5" t="s">
-        <v>12</v>
-      </c>
-      <c r="C5" t="s">
-        <v>28</v>
-      </c>
-      <c r="D5" t="s">
-        <v>26</v>
-      </c>
-      <c r="E5" t="s">
-        <v>26</v>
-      </c>
-      <c r="F5" t="s">
-        <v>27</v>
-      </c>
-      <c r="G5" t="n">
-        <v>15132516</v>
-      </c>
-      <c r="H5" t="b">
+        <v>22</v>
+      </c>
+      <c r="C5" t="n">
+        <v>1380155</v>
+      </c>
+      <c r="D5" t="b">
         <v>1</v>
       </c>
     </row>
@@ -1579,361 +1332,273 @@
   <dimension ref="A1"/>
   <sheetFormatPr defaultRowHeight="15.0" baseColWidth="10"/>
   <cols>
-    <col min="1" max="1" width="17.71" hidden="0" customWidth="1"/>
-    <col min="2" max="2" width="26.71" hidden="0" customWidth="1"/>
+    <col min="1" max="1" width="15.71" hidden="0" customWidth="1"/>
+    <col min="2" max="2" width="19.71" hidden="0" customWidth="1"/>
     <col min="3" max="3" width="136.71" hidden="0" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="s">
-        <v>45</v>
+        <v>38</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>46</v>
+        <v>39</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>47</v>
+        <v>40</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>48</v>
+        <v>41</v>
       </c>
       <c r="B2" t="s">
         <v>0</v>
       </c>
       <c r="C2" t="s">
-        <v>49</v>
+        <v>42</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>48</v>
+        <v>41</v>
       </c>
       <c r="B3" t="s">
         <v>1</v>
       </c>
       <c r="C3" t="s">
-        <v>50</v>
+        <v>43</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>48</v>
+        <v>41</v>
       </c>
       <c r="B4" t="s">
         <v>2</v>
       </c>
       <c r="C4" t="s">
-        <v>51</v>
+        <v>44</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>48</v>
+        <v>41</v>
       </c>
       <c r="B5" t="s">
         <v>3</v>
       </c>
       <c r="C5" t="s">
-        <v>52</v>
+        <v>45</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>48</v>
+        <v>41</v>
       </c>
       <c r="B6" t="s">
         <v>4</v>
       </c>
       <c r="C6" t="s">
-        <v>53</v>
+        <v>46</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="s">
-        <v>48</v>
+        <v>41</v>
       </c>
       <c r="B7" t="s">
         <v>5</v>
       </c>
       <c r="C7" t="s">
-        <v>54</v>
+        <v>47</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="s">
-        <v>48</v>
+        <v>41</v>
       </c>
       <c r="B8" t="s">
         <v>6</v>
       </c>
       <c r="C8" t="s">
-        <v>55</v>
+        <v>48</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="s">
-        <v>48</v>
+        <v>41</v>
       </c>
       <c r="B9" t="s">
         <v>7</v>
       </c>
       <c r="C9" t="s">
-        <v>56</v>
+        <v>49</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="s">
-        <v>48</v>
+        <v>41</v>
       </c>
       <c r="B10" t="s">
         <v>8</v>
       </c>
       <c r="C10" t="s">
-        <v>57</v>
+        <v>50</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="s">
-        <v>48</v>
+        <v>51</v>
       </c>
       <c r="B11" t="s">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="C11" t="s">
-        <v>58</v>
+        <v>42</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="s">
-        <v>48</v>
+        <v>51</v>
       </c>
       <c r="B12" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="C12" t="s">
-        <v>59</v>
+        <v>52</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="s">
-        <v>60</v>
+        <v>51</v>
       </c>
       <c r="B13" t="s">
-        <v>0</v>
+        <v>12</v>
       </c>
       <c r="C13" t="s">
-        <v>49</v>
+        <v>53</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="s">
-        <v>60</v>
+        <v>51</v>
       </c>
       <c r="B14" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C14" t="s">
-        <v>61</v>
+        <v>54</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="s">
-        <v>60</v>
+        <v>51</v>
       </c>
       <c r="B15" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C15" t="s">
-        <v>62</v>
+        <v>55</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="s">
-        <v>60</v>
+        <v>51</v>
       </c>
       <c r="B16" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="C16" t="s">
-        <v>63</v>
+        <v>56</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="s">
-        <v>60</v>
+        <v>51</v>
       </c>
       <c r="B17" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="C17" t="s">
-        <v>64</v>
+        <v>57</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="s">
-        <v>60</v>
+        <v>51</v>
       </c>
       <c r="B18" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="C18" t="s">
-        <v>65</v>
+        <v>58</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="s">
-        <v>60</v>
+        <v>51</v>
       </c>
       <c r="B19" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="C19" t="s">
-        <v>66</v>
+        <v>59</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="s">
+        <v>51</v>
+      </c>
+      <c r="B20" t="s">
+        <v>19</v>
+      </c>
+      <c r="C20" t="s">
         <v>60</v>
-      </c>
-      <c r="B20" t="s">
-        <v>20</v>
-      </c>
-      <c r="C20" t="s">
-        <v>67</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="B21" t="s">
-        <v>21</v>
+        <v>0</v>
       </c>
       <c r="C21" t="s">
-        <v>68</v>
+        <v>42</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="B22" t="s">
-        <v>22</v>
+        <v>15</v>
       </c>
       <c r="C22" t="s">
-        <v>69</v>
+        <v>56</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="B23" t="s">
-        <v>23</v>
+        <v>36</v>
       </c>
       <c r="C23" t="s">
-        <v>70</v>
+        <v>62</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="B24" t="s">
-        <v>24</v>
+        <v>37</v>
       </c>
       <c r="C24" t="s">
-        <v>71</v>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" t="s">
-        <v>72</v>
-      </c>
-      <c r="B25" t="s">
-        <v>0</v>
-      </c>
-      <c r="C25" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" t="s">
-        <v>72</v>
-      </c>
-      <c r="B26" t="s">
-        <v>42</v>
-      </c>
-      <c r="C26" t="s">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" t="s">
-        <v>72</v>
-      </c>
-      <c r="B27" t="s">
-        <v>20</v>
-      </c>
-      <c r="C27" t="s">
-        <v>67</v>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" t="s">
-        <v>72</v>
-      </c>
-      <c r="B28" t="s">
-        <v>16</v>
-      </c>
-      <c r="C28" t="s">
         <v>63</v>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" t="s">
-        <v>72</v>
-      </c>
-      <c r="B29" t="s">
-        <v>17</v>
-      </c>
-      <c r="C29" t="s">
-        <v>64</v>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" t="s">
-        <v>72</v>
-      </c>
-      <c r="B30" t="s">
-        <v>18</v>
-      </c>
-      <c r="C30" t="s">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" t="s">
-        <v>72</v>
-      </c>
-      <c r="B31" t="s">
-        <v>43</v>
-      </c>
-      <c r="C31" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" t="s">
-        <v>72</v>
-      </c>
-      <c r="B32" t="s">
-        <v>44</v>
-      </c>
-      <c r="C32" t="s">
-        <v>74</v>
       </c>
     </row>
   </sheetData>

</xml_diff>